<commit_message>
added log folder for debbuging
</commit_message>
<xml_diff>
--- a/test_data/product_info.xlsx
+++ b/test_data/product_info.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,17 +444,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Airpods Pro 2nd Gen Wireless Charging Bluetooth Headphone</t>
+          <t>Airpods Pro / tws wireless earbuds Bluetooth bluetooth headphone With High Base replica and long Battery</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>৳ 399</t>
+          <t>৳ 299</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Ratings 45</t>
+          <t>Ratings 999</t>
         </is>
       </c>
     </row>
@@ -464,17 +464,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Airpods Pro / tws wireless earbuds Bluetooth bluetooth headphone With High Base replica and long Battery</t>
+          <t>Leno~vo Livepods Airpods_Pro True Wireless Bluetooth Tws Headset Earbuds Earphones - Bluetooth Headphone</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>৳ 299</t>
+          <t>৳ 380</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Ratings 999</t>
+          <t>Ratings 18</t>
         </is>
       </c>
     </row>
@@ -484,17 +484,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Timack® D18 Wireless Headphones Bluetooth 5.2 Neckband Earphones Magnetic Sports Waterproof TWS Earbuds Headset with Microphone</t>
+          <t>Style Re TWS Bluetooth Earbuds - Wireless Earphones with ENC, Bass Boost, pro Battery, Type-C Charging - Charging Case - 3 Hours Playtime - Premium Sound Quality</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>৳ 323</t>
+          <t>৳ 263</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Ratings 1154</t>
+          <t>Ratings 1094</t>
         </is>
       </c>
     </row>
@@ -504,17 +504,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Timack® Y50 Air Buds Wireless Earbuds,TWS Bluetooth Earphone Wireless Headphones Stereo Bass Handsfree Gaming Headset with Charging Box Sports Bass In-Ear Earbuds, Immersive Deep Bass Air Buds</t>
+          <t>Mocho M10 TWS Earbuds 2500mAh Charging Box Bluetooth-compatible Stereo Waterproof</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>৳ 347</t>
+          <t>৳ 339</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ratings 107</t>
+          <t>Ratings 5484</t>
         </is>
       </c>
     </row>
@@ -524,17 +524,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Leno~vo Livepods Airpods_Pro True Wireless Bluetooth Tws Headset Earbuds Earphones - Bluetooth Headphone</t>
+          <t>Airpods Pro / tws Black edition wireless earbuds Bluetooth replica Bluetooth headphone</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>৳ 380</t>
+          <t>৳ 299</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Ratings 18</t>
+          <t>Ratings 76</t>
         </is>
       </c>
     </row>
@@ -544,17 +544,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Style Re TWS Bluetooth Earbuds - Wireless Earphones with ENC, Bass Boost, pro Battery, Type-C Charging - Charging Case - 3 Hours Playtime - Premium Sound Quality</t>
+          <t>AirPods Pro 2nd Generation Made in DUbai long lasting specials replica edition wireless blutooth Earbuds</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>৳ 263</t>
+          <t>৳ 309</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Ratings 1094</t>
+          <t>Ratings 81</t>
         </is>
       </c>
     </row>
@@ -564,17 +564,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Airpods Pro / tws Black edition wireless earbuds Bluetooth replica Bluetooth headphone</t>
+          <t>AirPods Pro 2nd Generation long lasting specials edition wireless Blutooth replica Earbuds By Next Gadget</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>৳ 299</t>
+          <t>৳ 309</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Ratings 76</t>
+          <t>Ratings 357</t>
         </is>
       </c>
     </row>
@@ -584,17 +584,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AirPods Pro 2nd Generation Made in DUbai long lasting specials replica edition wireless blutooth Earbuds</t>
+          <t>M10 TWS Earbuds 2500mAh Charging Box Bluetooth-compatible Stereo Waterproof</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>৳ 309</t>
+          <t>৳ 316</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Ratings 81</t>
+          <t>Ratings 6</t>
         </is>
       </c>
     </row>
@@ -604,137 +604,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Airpods Pro / tws wireless earbuds Bluetooth bluetooth headphone With High Base and long Battery</t>
+          <t>AirPods Pro 2nd genaration Made in Dubai Wireless Charging Bluetooth Earbuds</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>৳ 295</t>
+          <t>৳ 457</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Ratings 142</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>AirPods Pro 2nd Generation long lasting specials edition wireless Blutooth replica Earbuds By Next Gadget</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>৳ 309</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Ratings 357</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Timack® N35 TWS Gaming Earbuds Low Latency Bluetooth Earphones Stereo Wireless 5.1 Bluetooth Headphones Touch Control Headset</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>৳ 622</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Ratings 215</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>M28 TWS Bluetooth 5.1 Gaming Headset Dual Mode Wireless Earphones Sports Stereo Sound Low Latency LED Digital Display Smart Touch Earphone</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>৳ 499</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Ratings 666</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>M19 Wireless Earbuds 5.1 Bluetooth Headphones Touch Control with Wireless Charging Case IPX8 Waterproof TWS Stereo Earphones in-Ear Built-in Mic Headset</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>৳ 286</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>No Ratings</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>M19 Earbuds TWS Touch Control Wireless Bluetooth 5.1 Headphones With Microphone With flashlight</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>৳ 279</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Ratings 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Timack® X15 Gaming Earbuds Wireless Earphone Bluetooth 5.0 Low Latency Stereo Bass Handsfree, Touch Control Noise Cancelling Wireless Headphone with Microphone</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>৳ 372</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Ratings 82</t>
+          <t>Ratings 911</t>
         </is>
       </c>
     </row>

</xml_diff>